<commit_message>
changes for publication of DeID Handbook 2.0.0
</commit_message>
<xml_diff>
--- a/ITI/DeId/CodeSystem-DeIdentificationEntityType.xlsx
+++ b/ITI/DeId/CodeSystem-DeIdentificationEntityType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>2.0.0-comment</t>
+    <t>2.0.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-12T10:54:51-05:00</t>
+    <t>2026-10-17T19:18:20-05:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>